<commit_message>
Update logic for AT
</commit_message>
<xml_diff>
--- a/data/Mar/Bảng-đối-soát-t3-2026.xlsx
+++ b/data/Mar/Bảng-đối-soát-t3-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Mar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E6C78B-B386-447D-BEDC-C00391C75760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E458806-5293-4F5E-9B46-94AC8182F15F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="12" xr2:uid="{7DBF314D-BB0B-41C9-BACA-A4F738DC8062}"/>
   </bookViews>
@@ -55,6 +55,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>

</xml_diff>